<commit_message>
Updated with the columns fixed.
</commit_message>
<xml_diff>
--- a/docs/tricorder_parts.xlsx
+++ b/docs/tricorder_parts.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="76">
   <si>
     <t xml:space="preserve">Category</t>
   </si>
@@ -61,6 +61,9 @@
     <t xml:space="preserve">Adafruit BME688 #5046 (gas+temp+RH+pressure, I2C)</t>
   </si>
   <si>
+    <t xml:space="preserve">VERIFIED DigiKey Jul 2026</t>
+  </si>
+  <si>
     <t xml:space="preserve">https://www.adafruit.com/product/5046</t>
   </si>
   <si>
@@ -73,6 +76,9 @@
     <t xml:space="preserve">Adafruit SCD-41 #5190 (true CO2, NDIR, I2C)</t>
   </si>
   <si>
+    <t xml:space="preserve">ESTIMATE - not captured this session</t>
+  </si>
+  <si>
     <t xml:space="preserve">https://www.adafruit.com/product/5190</t>
   </si>
   <si>
@@ -145,6 +151,9 @@
     <t xml:space="preserve">AD9226 ADC module, 12-bit 65 MS/s parallel, Pmod form</t>
   </si>
   <si>
+    <t xml:space="preserve">ESTIMATE - generic ~$10-30</t>
+  </si>
+  <si>
     <t xml:space="preserve">https://fraserinnovations.com/product/fii-bd9226-high-speed-ad-module-12-digital-65mhz-data-sampling-ad9226/</t>
   </si>
   <si>
@@ -157,6 +166,9 @@
     <t xml:space="preserve">AD9708 DAC module, 8-bit 125 MS/s (often AD9280+AD9708 combo)</t>
   </si>
   <si>
+    <t xml:space="preserve">ESTIMATE - ~$15-25</t>
+  </si>
+  <si>
     <t xml:space="preserve">https://www.ebay.com/sch/i.html?_nkw=AD9708+module</t>
   </si>
   <si>
@@ -172,6 +184,9 @@
     <t xml:space="preserve">OV7670 camera module (8-bit DVP, 640x480@30fps)</t>
   </si>
   <si>
+    <t xml:space="preserve">ESTIMATE - ~$5-12</t>
+  </si>
+  <si>
     <t xml:space="preserve">https://www.amazon.com/ov7670-camera-module/s?k=ov7670+camera+module</t>
   </si>
   <si>
@@ -187,6 +202,9 @@
     <t xml:space="preserve">SiPM module (onsemi MICROFC-SMA-10035-GEVB eval)</t>
   </si>
   <si>
+    <t xml:space="preserve">ESTIMATE - unverified; hobby SiPM $30-60 AliExpress</t>
+  </si>
+  <si>
     <t xml:space="preserve">https://www.digikey.com/en/products/detail/onsemi/MICROFC-SMA-10035-GEVB/6220699</t>
   </si>
   <si>
@@ -199,6 +217,9 @@
     <t xml:space="preserve">AD8332 VGA board (ultrasound AFE)</t>
   </si>
   <si>
+    <t xml:space="preserve">ESTIMATE - ~$25-40</t>
+  </si>
+  <si>
     <t xml:space="preserve">https://www.ebay.com/sch/i.html?_nkw=AD8332+module</t>
   </si>
   <si>
@@ -209,6 +230,9 @@
   </si>
   <si>
     <t xml:space="preserve">Piezo ultrasonic transducers, 40 kHz pair (TX/RX)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ESTIMATE</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.amazon.com/s?k=40khz+ultrasonic+transducer+piezo</t>
@@ -347,11 +371,15 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -388,15 +416,15 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -655,433 +683,457 @@
   <dimension ref="A1:J17"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="44"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="44"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+    <row r="2" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D2" s="2" t="n">
+      <c r="D2" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="E2" s="4" t="n">
+      <c r="E2" s="5" t="n">
         <v>31.11</v>
       </c>
-      <c r="F2" s="5" t="n">
+      <c r="F2" s="6" t="n">
         <f aca="false">D2*E2</f>
         <v>31.11</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="G2" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="H2" s="3" t="s">
+      <c r="H2" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="I2" s="3" t="s">
+      <c r="I2" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="J2" s="3"/>
-    </row>
-    <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+      <c r="J2" s="4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C3" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="D3" s="2" t="n">
+      <c r="C3" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D3" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="E3" s="4" t="n">
+      <c r="E3" s="5" t="n">
         <v>49.5</v>
       </c>
-      <c r="F3" s="5" t="n">
+      <c r="F3" s="6" t="n">
         <f aca="false">D3*E3</f>
         <v>49.5</v>
       </c>
-      <c r="G3" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="H3" s="3" t="s">
+      <c r="G3" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="I3" s="3" t="s">
+      <c r="H3" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="J3" s="3"/>
-    </row>
-    <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
+      <c r="I3" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="J3" s="4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C4" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="D4" s="2" t="n">
+      <c r="C4" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D4" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="E4" s="4" t="n">
+      <c r="E4" s="5" t="n">
         <v>7.24</v>
       </c>
-      <c r="F4" s="5" t="n">
+      <c r="F4" s="6" t="n">
         <f aca="false">D4*E4</f>
         <v>7.24</v>
       </c>
-      <c r="G4" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="I4" s="3" t="s">
+      <c r="G4" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H4" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="J4" s="3"/>
-    </row>
-    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="s">
+      <c r="I4" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="D5" s="2" t="n">
+      <c r="C5" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="D5" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="E5" s="4" t="n">
+      <c r="E5" s="5" t="n">
         <v>15.95</v>
       </c>
-      <c r="F5" s="5" t="n">
+      <c r="F5" s="6" t="n">
         <f aca="false">D5*E5</f>
         <v>15.95</v>
       </c>
-      <c r="G5" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>26</v>
-      </c>
-      <c r="I5" s="3" t="s">
+      <c r="G5" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="H5" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="J5" s="3"/>
-    </row>
-    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="s">
+      <c r="I5" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="J5" s="4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="D6" s="2" t="n">
+      <c r="C6" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D6" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="E6" s="4" t="n">
+      <c r="E6" s="5" t="n">
         <v>4.95</v>
       </c>
-      <c r="F6" s="5" t="n">
+      <c r="F6" s="6" t="n">
         <f aca="false">D6*E6</f>
         <v>29.7</v>
       </c>
-      <c r="G6" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="H6" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="I6" s="3" t="s">
+      <c r="G6" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="H6" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="J6" s="3"/>
-    </row>
-    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="6" t="s">
+      <c r="I6" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="J6" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="C7" s="7" t="s">
+    </row>
+    <row r="7" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="D7" s="6" t="n">
+      <c r="B7" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="C7" s="8" t="s">
+        <v>37</v>
+      </c>
+      <c r="D7" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="E7" s="8" t="n">
+      <c r="E7" s="9" t="n">
         <v>19.5</v>
       </c>
-      <c r="F7" s="9" t="n">
+      <c r="F7" s="10" t="n">
         <f aca="false">D7*E7</f>
         <v>19.5</v>
       </c>
-      <c r="G7" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="H7" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="I7" s="7" t="s">
+      <c r="G7" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="H7" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="J7" s="7"/>
-    </row>
-    <row r="8" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="B8" s="6" t="s">
+      <c r="I7" s="8" t="s">
         <v>39</v>
       </c>
-      <c r="C8" s="7" t="s">
+      <c r="J7" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="D8" s="6" t="n">
+    </row>
+    <row r="8" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="C8" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="D8" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="E8" s="8" t="n">
+      <c r="E8" s="9" t="n">
         <v>25</v>
       </c>
-      <c r="F8" s="9" t="n">
+      <c r="F8" s="10" t="n">
         <f aca="false">D8*E8</f>
         <v>25</v>
       </c>
-      <c r="G8" s="7" t="s">
+      <c r="G8" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="H8" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="I8" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="J8" s="8" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B9" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="H8" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="I8" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="J8" s="7"/>
-    </row>
-    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="C9" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="D9" s="6" t="n">
+      <c r="C9" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="D9" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="E9" s="8" t="n">
+      <c r="E9" s="9" t="n">
         <v>20</v>
       </c>
-      <c r="F9" s="9" t="n">
+      <c r="F9" s="10" t="n">
         <f aca="false">D9*E9</f>
         <v>20</v>
       </c>
-      <c r="G9" s="7" t="s">
-        <v>45</v>
-      </c>
-      <c r="H9" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="I9" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="J9" s="7"/>
-    </row>
-    <row r="10" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="B10" s="6" t="s">
+      <c r="G9" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="C10" s="7" t="s">
+      <c r="H9" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="D10" s="6" t="n">
+      <c r="I9" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="J9" s="8" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="D10" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="E10" s="8" t="n">
+      <c r="E10" s="9" t="n">
         <v>8</v>
       </c>
-      <c r="F10" s="9" t="n">
+      <c r="F10" s="10" t="n">
         <f aca="false">D10*E10</f>
         <v>8</v>
       </c>
-      <c r="G10" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="H10" s="7" t="s">
-        <v>51</v>
-      </c>
-      <c r="I10" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="J10" s="7"/>
-    </row>
-    <row r="11" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="C11" s="7" t="s">
+      <c r="G10" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="D11" s="6" t="n">
+      <c r="H10" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="I10" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="J10" s="8" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="C11" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="D11" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="E11" s="8" t="n">
+      <c r="E11" s="9" t="n">
         <v>150</v>
       </c>
-      <c r="F11" s="9" t="n">
+      <c r="F11" s="10" t="n">
         <f aca="false">D11*E11</f>
         <v>150</v>
       </c>
-      <c r="G11" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="H11" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="I11" s="7" t="s">
-        <v>57</v>
-      </c>
-      <c r="J11" s="7"/>
-    </row>
-    <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="B12" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="C12" s="7" t="s">
-        <v>58</v>
-      </c>
-      <c r="D12" s="6" t="n">
+      <c r="G11" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="H11" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="I11" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="J11" s="8" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="C12" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="D12" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="E12" s="8" t="n">
+      <c r="E12" s="9" t="n">
         <v>30</v>
       </c>
-      <c r="F12" s="9" t="n">
+      <c r="F12" s="10" t="n">
         <f aca="false">D12*E12</f>
         <v>30</v>
       </c>
-      <c r="G12" s="7" t="s">
-        <v>59</v>
-      </c>
-      <c r="H12" s="7" t="s">
-        <v>60</v>
-      </c>
-      <c r="I12" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="J12" s="7"/>
-    </row>
-    <row r="13" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="B13" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="C13" s="7" t="s">
-        <v>62</v>
-      </c>
-      <c r="D13" s="6" t="n">
+      <c r="G12" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="H12" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="I12" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="J12" s="8" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="C13" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="D13" s="7" t="n">
         <v>2</v>
       </c>
-      <c r="E13" s="8" t="n">
+      <c r="E13" s="9" t="n">
         <v>3</v>
       </c>
-      <c r="F13" s="9" t="n">
+      <c r="F13" s="10" t="n">
         <f aca="false">D13*E13</f>
         <v>6</v>
       </c>
-      <c r="G13" s="7" t="s">
-        <v>63</v>
-      </c>
-      <c r="H13" s="7" t="s">
-        <v>64</v>
-      </c>
-      <c r="I13" s="7" t="s">
-        <v>65</v>
-      </c>
-      <c r="J13" s="7"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C15" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="F15" s="11" t="n">
+      <c r="G13" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="H13" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="I13" s="8" t="s">
+        <v>72</v>
+      </c>
+      <c r="J13" s="8" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C15" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="F15" s="12" t="n">
         <f aca="false">SUM(F2:F13)</f>
         <v>392</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="12" t="s">
-        <v>67</v>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="13" t="s">
+        <v>75</v>
       </c>
     </row>
   </sheetData>

</xml_diff>